<commit_message>
chore: Remove README and DESCRIPTION documentation files
- Delete DESCRIPTION.md (project overview)
- Delete README.md (comprehensive user guide and setup instructions)
- Update JIRA_template.xlsx with template refinements
- Modify app.py, create_template.py, and related dashboard files
- Consolidate documentation into single source of truth or migrate to alternative format
</commit_message>
<xml_diff>
--- a/JIRA_template.xlsx
+++ b/JIRA_template.xlsx
@@ -11,7 +11,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Instructions" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'JIRA Data'!$A$1:$S$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'JIRA Data'!$A$1:$U$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -489,122 +489,134 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S11"/>
+  <dimension ref="A1:U11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="10" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="20" customWidth="1" min="4" max="4"/>
-    <col width="36" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="9" customWidth="1" min="7" max="7"/>
-    <col width="15" customWidth="1" min="8" max="8"/>
-    <col width="16" customWidth="1" min="9" max="9"/>
-    <col width="17" customWidth="1" min="10" max="10"/>
-    <col width="15" customWidth="1" min="11" max="11"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="36" customWidth="1" min="6" max="6"/>
+    <col width="30" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="15" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
     <col width="15" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="13" customWidth="1" min="14" max="14"/>
+    <col width="15" customWidth="1" min="13" max="13"/>
+    <col width="14" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
-    <col width="10" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="13" customWidth="1" min="18" max="18"/>
-    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="16" max="16"/>
+    <col width="13" customWidth="1" min="17" max="17"/>
+    <col width="10" customWidth="1" min="18" max="18"/>
+    <col width="12" customWidth="1" min="19" max="19"/>
+    <col width="13" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="21" max="21"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Client</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>Project</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>Sprint</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>EPIC</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>Quality</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>Budget Planned</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>Budget Consumed</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>Budget Remaining</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Saving Planned</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>Saving Achived</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>Saving Pending</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>Start Date</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>Date</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>Story Points</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>Priority</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>Assignee</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>Status</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>Dependencies</t>
         </is>
@@ -613,498 +625,548 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D2" s="2" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>User Auth</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
         <is>
           <t>Login with SSO</t>
         </is>
       </c>
-      <c r="F2" s="2" t="inlineStr">
+      <c r="G2" s="2" t="inlineStr">
         <is>
           <t>Frontend implementation</t>
         </is>
       </c>
-      <c r="G2" s="3" t="n">
+      <c r="H2" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H2" s="3" t="n">
+      <c r="I2" s="3" t="n">
         <v>3000</v>
       </c>
-      <c r="I2" s="3" t="n">
+      <c r="J2" s="3" t="n">
         <v>1800</v>
       </c>
-      <c r="J2" s="3" t="n">
+      <c r="K2" s="3" t="n">
         <v>1200</v>
       </c>
-      <c r="K2" s="3" t="n">
+      <c r="L2" s="3" t="n">
         <v>400</v>
-      </c>
-      <c r="L2" s="3" t="n">
-        <v>200</v>
       </c>
       <c r="M2" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="N2" s="4" t="n">
+      <c r="N2" s="3" t="n">
+        <v>200</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>46027</v>
+      </c>
+      <c r="P2" s="4" t="n">
         <v>46032</v>
       </c>
-      <c r="O2" s="3" t="n">
+      <c r="Q2" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="R2" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="Q2" s="2" t="inlineStr">
+      <c r="S2" s="2" t="inlineStr">
         <is>
           <t>Alice</t>
         </is>
       </c>
-      <c r="R2" s="2" t="inlineStr">
+      <c r="T2" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="S2" s="2" t="inlineStr"/>
+      <c r="U2" s="2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="5" t="inlineStr">
         <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="B3" s="5" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="C3" s="5" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="D3" s="5" t="inlineStr">
         <is>
           <t>Sprint 1</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="E3" s="5" t="inlineStr">
         <is>
           <t>User Auth</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="F3" s="5" t="inlineStr">
         <is>
           <t>Login with SSO</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="G3" s="5" t="inlineStr">
         <is>
           <t>Unit tests</t>
         </is>
       </c>
-      <c r="G3" s="6" t="n">
+      <c r="H3" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="6" t="n">
+      <c r="I3" s="6" t="n">
         <v>1200</v>
       </c>
-      <c r="I3" s="6" t="n">
+      <c r="J3" s="6" t="n">
         <v>900</v>
       </c>
-      <c r="J3" s="6" t="n">
+      <c r="K3" s="6" t="n">
         <v>300</v>
       </c>
-      <c r="K3" s="6" t="n">
+      <c r="L3" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="L3" s="6" t="n">
+      <c r="M3" s="6" t="n">
         <v>90</v>
       </c>
-      <c r="M3" s="6" t="n">
+      <c r="N3" s="6" t="n">
         <v>60</v>
       </c>
-      <c r="N3" s="7" t="n">
+      <c r="O3" s="7" t="n">
+        <v>46030</v>
+      </c>
+      <c r="P3" s="7" t="n">
         <v>46036</v>
       </c>
-      <c r="O3" s="6" t="n">
+      <c r="Q3" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="P3" s="5" t="inlineStr">
+      <c r="R3" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="Q3" s="5" t="inlineStr">
+      <c r="S3" s="5" t="inlineStr">
         <is>
           <t>Bob</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="T3" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr"/>
+      <c r="U3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>Acme Corp</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="D4" s="2" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>User Auth</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
         <is>
           <t>Password reset flow</t>
         </is>
       </c>
-      <c r="F4" s="2" t="inlineStr">
+      <c r="G4" s="2" t="inlineStr">
         <is>
           <t>API endpoint</t>
         </is>
       </c>
-      <c r="G4" s="3" t="n">
+      <c r="H4" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="H4" s="3" t="n">
-        <v>2500</v>
       </c>
       <c r="I4" s="3" t="n">
         <v>2500</v>
       </c>
       <c r="J4" s="3" t="n">
+        <v>2500</v>
+      </c>
+      <c r="K4" s="3" t="n">
         <v>0</v>
-      </c>
-      <c r="K4" s="3" t="n">
-        <v>300</v>
       </c>
       <c r="L4" s="3" t="n">
         <v>300</v>
       </c>
       <c r="M4" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="N4" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="4" t="n">
+      <c r="O4" s="4" t="n">
+        <v>46042</v>
+      </c>
+      <c r="P4" s="4" t="n">
         <v>46050</v>
       </c>
-      <c r="O4" s="3" t="n">
+      <c r="Q4" s="3" t="n">
         <v>5</v>
       </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="R4" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="Q4" s="2" t="inlineStr">
+      <c r="S4" s="2" t="inlineStr">
         <is>
           <t>Carol</t>
         </is>
       </c>
-      <c r="R4" s="2" t="inlineStr">
+      <c r="T4" s="2" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="S4" s="2" t="inlineStr"/>
+      <c r="U4" s="2" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
+          <t>Beta Ltd</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="C5" s="5" t="inlineStr">
         <is>
           <t>Alpha</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Sprint 2</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>User Auth</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="F5" s="5" t="inlineStr">
         <is>
           <t>Password reset flow</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="G5" s="5" t="inlineStr">
         <is>
           <t>Email template design</t>
         </is>
       </c>
-      <c r="G5" s="6" t="n">
+      <c r="H5" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H5" s="6" t="n">
+      <c r="I5" s="6" t="n">
         <v>800</v>
-      </c>
-      <c r="I5" s="6" t="n">
-        <v>400</v>
       </c>
       <c r="J5" s="6" t="n">
         <v>400</v>
       </c>
       <c r="K5" s="6" t="n">
+        <v>400</v>
+      </c>
+      <c r="L5" s="6" t="n">
         <v>100</v>
-      </c>
-      <c r="L5" s="6" t="n">
-        <v>50</v>
       </c>
       <c r="M5" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="N5" s="7" t="n">
+      <c r="N5" s="6" t="n">
+        <v>50</v>
+      </c>
+      <c r="O5" s="7" t="n">
+        <v>46047</v>
+      </c>
+      <c r="P5" s="7" t="n">
         <v>46057</v>
       </c>
-      <c r="O5" s="6" t="n">
+      <c r="Q5" s="6" t="n">
         <v>1</v>
       </c>
-      <c r="P5" s="5" t="inlineStr">
+      <c r="R5" s="5" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
       </c>
-      <c r="Q5" s="5" t="inlineStr">
+      <c r="S5" s="5" t="inlineStr">
         <is>
           <t>Dave</t>
         </is>
       </c>
-      <c r="R5" s="5" t="inlineStr">
+      <c r="T5" s="5" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="S5" s="5" t="inlineStr"/>
+      <c r="U5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>Beta Ltd</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B6" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="C6" s="2" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="D6" s="2" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Reporting</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>Management dashboard</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Data model</t>
         </is>
       </c>
-      <c r="G6" s="3" t="n">
+      <c r="H6" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="H6" s="3" t="n">
+      <c r="I6" s="3" t="n">
         <v>5000</v>
       </c>
-      <c r="I6" s="3" t="n">
+      <c r="J6" s="3" t="n">
         <v>3000</v>
       </c>
-      <c r="J6" s="3" t="n">
+      <c r="K6" s="3" t="n">
         <v>2000</v>
       </c>
-      <c r="K6" s="3" t="n">
+      <c r="L6" s="3" t="n">
         <v>600</v>
-      </c>
-      <c r="L6" s="3" t="n">
-        <v>300</v>
       </c>
       <c r="M6" s="3" t="n">
         <v>300</v>
       </c>
-      <c r="N6" s="4" t="n">
+      <c r="N6" s="3" t="n">
+        <v>300</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>46058</v>
+      </c>
+      <c r="P6" s="4" t="n">
         <v>46064</v>
       </c>
-      <c r="O6" s="3" t="n">
+      <c r="Q6" s="3" t="n">
         <v>8</v>
       </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="R6" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="Q6" s="2" t="inlineStr">
+      <c r="S6" s="2" t="inlineStr">
         <is>
           <t>Eve</t>
         </is>
       </c>
-      <c r="R6" s="2" t="inlineStr">
+      <c r="T6" s="2" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="S6" s="2" t="inlineStr"/>
+      <c r="U6" s="2" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>Gamma Inc</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="C7" s="5" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="D7" s="5" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="E7" s="5" t="inlineStr">
         <is>
           <t>Reporting</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="F7" s="5" t="inlineStr">
         <is>
           <t>Management dashboard</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="G7" s="5" t="inlineStr">
         <is>
           <t>Chart components</t>
         </is>
       </c>
-      <c r="G7" s="6" t="n">
+      <c r="H7" s="6" t="n">
         <v>2</v>
       </c>
-      <c r="H7" s="6" t="n">
+      <c r="I7" s="6" t="n">
         <v>2200</v>
-      </c>
-      <c r="I7" s="6" t="n">
-        <v>1100</v>
       </c>
       <c r="J7" s="6" t="n">
         <v>1100</v>
       </c>
       <c r="K7" s="6" t="n">
+        <v>1100</v>
+      </c>
+      <c r="L7" s="6" t="n">
         <v>250</v>
       </c>
-      <c r="L7" s="6" t="n">
+      <c r="M7" s="6" t="n">
         <v>100</v>
       </c>
-      <c r="M7" s="6" t="n">
+      <c r="N7" s="6" t="n">
         <v>150</v>
       </c>
-      <c r="N7" s="7" t="n">
+      <c r="O7" s="7" t="n">
+        <v>46063</v>
+      </c>
+      <c r="P7" s="7" t="n">
         <v>46071</v>
       </c>
-      <c r="O7" s="6" t="n">
+      <c r="Q7" s="6" t="n">
         <v>3</v>
       </c>
-      <c r="P7" s="5" t="inlineStr">
+      <c r="R7" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="Q7" s="5" t="inlineStr">
+      <c r="S7" s="5" t="inlineStr">
         <is>
           <t>Frank</t>
         </is>
       </c>
-      <c r="R7" s="5" t="inlineStr">
+      <c r="T7" s="5" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="S7" s="5" t="inlineStr"/>
+      <c r="U7" s="5" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Gamma Inc</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
           <t>Bug</t>
         </is>
       </c>
-      <c r="B8" s="2" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="C8" s="2" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Sprint 3</t>
         </is>
       </c>
-      <c r="D8" s="2" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Reporting</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
         <is>
           <t>Management dashboard</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
+      <c r="G8" s="2" t="inlineStr">
         <is>
           <t>Fix date filter</t>
         </is>
       </c>
-      <c r="G8" s="3" t="n">
+      <c r="H8" s="3" t="n">
         <v>3</v>
       </c>
-      <c r="H8" s="3" t="n">
+      <c r="I8" s="3" t="n">
         <v>600</v>
       </c>
-      <c r="I8" s="3" t="n">
+      <c r="J8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="J8" s="3" t="n">
+      <c r="K8" s="3" t="n">
         <v>600</v>
-      </c>
-      <c r="K8" s="3" t="n">
-        <v>0</v>
       </c>
       <c r="L8" s="3" t="n">
         <v>0</v>
@@ -1112,264 +1174,294 @@
       <c r="M8" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="N8" s="4" t="n">
+      <c r="N8" s="3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>46068</v>
+      </c>
+      <c r="P8" s="4" t="n">
         <v>46073</v>
       </c>
-      <c r="O8" s="3" t="n">
+      <c r="Q8" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="R8" s="2" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="Q8" s="2" t="inlineStr">
+      <c r="S8" s="2" t="inlineStr">
         <is>
           <t>Grace</t>
         </is>
       </c>
-      <c r="R8" s="2" t="inlineStr">
+      <c r="T8" s="2" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="S8" s="2" t="inlineStr"/>
+      <c r="U8" s="2" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
+          <t>Delta Co</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="C9" s="5" t="inlineStr">
         <is>
           <t>Beta</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="D9" s="5" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="E9" s="5" t="inlineStr">
         <is>
           <t>Integrations</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
+      <c r="F9" s="5" t="inlineStr">
         <is>
           <t>Connect to third-party API</t>
         </is>
       </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="G9" s="5" t="inlineStr">
         <is>
           <t>OAuth handshake</t>
         </is>
       </c>
-      <c r="G9" s="6" t="n">
+      <c r="H9" s="6" t="n">
         <v>0</v>
-      </c>
-      <c r="H9" s="6" t="n">
-        <v>4000</v>
       </c>
       <c r="I9" s="6" t="n">
         <v>4000</v>
       </c>
       <c r="J9" s="6" t="n">
+        <v>4000</v>
+      </c>
+      <c r="K9" s="6" t="n">
         <v>0</v>
-      </c>
-      <c r="K9" s="6" t="n">
-        <v>500</v>
       </c>
       <c r="L9" s="6" t="n">
         <v>500</v>
       </c>
       <c r="M9" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="N9" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="7" t="n">
+      <c r="O9" s="7" t="n">
+        <v>46081</v>
+      </c>
+      <c r="P9" s="7" t="n">
         <v>46086</v>
       </c>
-      <c r="O9" s="6" t="n">
+      <c r="Q9" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="P9" s="5" t="inlineStr">
+      <c r="R9" s="5" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="Q9" s="5" t="inlineStr">
+      <c r="S9" s="5" t="inlineStr">
         <is>
           <t>Henry</t>
         </is>
       </c>
-      <c r="R9" s="5" t="inlineStr">
+      <c r="T9" s="5" t="inlineStr">
         <is>
           <t>Done</t>
         </is>
       </c>
-      <c r="S9" s="5" t="inlineStr"/>
+      <c r="U9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>Delta Co</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
           <t>Task</t>
         </is>
       </c>
-      <c r="B10" s="2" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Gamma</t>
         </is>
       </c>
-      <c r="C10" s="2" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Sprint 4</t>
         </is>
       </c>
-      <c r="D10" s="2" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Integrations</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
         <is>
           <t>Connect to third-party API</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
+      <c r="G10" s="2" t="inlineStr">
         <is>
           <t>Rate-limit handling</t>
         </is>
       </c>
-      <c r="G10" s="3" t="n">
+      <c r="H10" s="3" t="n">
         <v>1</v>
       </c>
-      <c r="H10" s="3" t="n">
+      <c r="I10" s="3" t="n">
         <v>1500</v>
-      </c>
-      <c r="I10" s="3" t="n">
-        <v>750</v>
       </c>
       <c r="J10" s="3" t="n">
         <v>750</v>
       </c>
       <c r="K10" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="L10" s="3" t="n">
         <v>200</v>
       </c>
-      <c r="L10" s="3" t="n">
+      <c r="M10" s="3" t="n">
         <v>80</v>
       </c>
-      <c r="M10" s="3" t="n">
+      <c r="N10" s="3" t="n">
         <v>120</v>
       </c>
-      <c r="N10" s="4" t="n">
+      <c r="O10" s="4" t="n">
+        <v>46086</v>
+      </c>
+      <c r="P10" s="4" t="n">
         <v>46093</v>
       </c>
-      <c r="O10" s="3" t="n">
+      <c r="Q10" s="3" t="n">
         <v>2</v>
       </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="R10" s="2" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="Q10" s="2" t="inlineStr">
+      <c r="S10" s="2" t="inlineStr">
         <is>
           <t>Iris</t>
         </is>
       </c>
-      <c r="R10" s="2" t="inlineStr">
+      <c r="T10" s="2" t="inlineStr">
         <is>
           <t>In Progress</t>
         </is>
       </c>
-      <c r="S10" s="2" t="inlineStr"/>
+      <c r="U10" s="2" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
+          <t>Epsilon LLC</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr">
+        <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="C11" s="5" t="inlineStr">
         <is>
           <t>Gamma</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="D11" s="5" t="inlineStr">
         <is>
           <t>Sprint 5</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="E11" s="5" t="inlineStr">
         <is>
           <t>Performance</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="F11" s="5" t="inlineStr">
         <is>
           <t>Reduce API response time</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="G11" s="5" t="inlineStr">
         <is>
           <t>Query optimisation</t>
         </is>
       </c>
-      <c r="G11" s="6" t="n">
+      <c r="H11" s="6" t="n">
         <v>0</v>
       </c>
-      <c r="H11" s="6" t="n">
+      <c r="I11" s="6" t="n">
         <v>3500</v>
       </c>
-      <c r="I11" s="6" t="n">
+      <c r="J11" s="6" t="n">
         <v>500</v>
       </c>
-      <c r="J11" s="6" t="n">
+      <c r="K11" s="6" t="n">
         <v>3000</v>
       </c>
-      <c r="K11" s="6" t="n">
+      <c r="L11" s="6" t="n">
         <v>450</v>
       </c>
-      <c r="L11" s="6" t="n">
+      <c r="M11" s="6" t="n">
         <v>50</v>
       </c>
-      <c r="M11" s="6" t="n">
+      <c r="N11" s="6" t="n">
         <v>400</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="O11" s="7" t="n">
+        <v>46091</v>
+      </c>
+      <c r="P11" s="7" t="n">
         <v>46100</v>
       </c>
-      <c r="O11" s="6" t="n">
+      <c r="Q11" s="6" t="n">
         <v>5</v>
       </c>
-      <c r="P11" s="5" t="inlineStr">
+      <c r="R11" s="5" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="Q11" s="5" t="inlineStr">
+      <c r="S11" s="5" t="inlineStr">
         <is>
           <t>Jack</t>
         </is>
       </c>
-      <c r="R11" s="5" t="inlineStr">
+      <c r="T11" s="5" t="inlineStr">
         <is>
           <t>To Do</t>
         </is>
       </c>
-      <c r="S11" s="5" t="inlineStr"/>
+      <c r="U11" s="5" t="inlineStr"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:S1"/>
+  <autoFilter ref="A1:U1"/>
   <dataValidations count="3">
-    <dataValidation sqref="A2:A210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="B2:B210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Story,Task,Bug,Sub-task,Epic"</formula1>
     </dataValidation>
-    <dataValidation sqref="P2:P210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="R2:R210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"High,Medium,Low,Critical"</formula1>
     </dataValidation>
-    <dataValidation sqref="R2:R210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="T2:T210" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"To Do,In Progress,Done,Blocked,In Review"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1383,7 +1475,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A28"/>
+  <dimension ref="A1:A30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="90" customWidth="1" min="1" max="1"/>
@@ -1409,169 +1501,183 @@
     <row r="4">
       <c r="A4" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Type            — Ticket type: Story, Task, Bug, Sub-task, Epic</t>
+          <t xml:space="preserve">  Client          — Client or customer name (e.g. Acme Corp, Beta Ltd)</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Project         — Project key or name (e.g. Alpha, Beta)</t>
+          <t xml:space="preserve">  Type            — Ticket type: Story, Task, Bug, Sub-task, Epic</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Sprint          — Sprint name (e.g. Sprint 1)</t>
+          <t xml:space="preserve">  Project         — Project key or name (e.g. Alpha, Beta)</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  EPIC            — Epic name the ticket belongs to</t>
+          <t xml:space="preserve">  Sprint          — Sprint name (e.g. Sprint 1)</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Story           — Parent story description</t>
+          <t xml:space="preserve">  EPIC            — Epic name the ticket belongs to</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Task            — Task description</t>
+          <t xml:space="preserve">  Story           — Parent story description</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Quality         — Integer quality score (0 = no issues)</t>
+          <t xml:space="preserve">  Task            — Task description</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Budget Planned  — Planned budget in your currency</t>
+          <t xml:space="preserve">  Quality         — Integer quality score (0 = no issues)</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Budget Consumed — Budget spent so far</t>
+          <t xml:space="preserve">  Budget Planned  — Planned budget in your currency</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Budget Remaining— Remaining budget (can be formula = Planned - Consumed)</t>
+          <t xml:space="preserve">  Budget Consumed — Budget spent so far</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Saving Planned  — Planned savings</t>
+          <t xml:space="preserve">  Budget Remaining— Remaining budget (can be formula = Planned - Consumed)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Saving Achived  — Achieved savings (note: keep original spelling)</t>
+          <t xml:space="preserve">  Saving Planned  — Planned savings</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Saving Pending  — Pending savings</t>
+          <t xml:space="preserve">  Saving Achived  — Achieved savings (note: keep original spelling)</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Date            — Date in YYYY-MM-DD format</t>
+          <t xml:space="preserve">  Saving Pending  — Pending savings</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Story Points    — Effort estimate (integer)</t>
+          <t xml:space="preserve">  Start Date      — Task start date in YYYY-MM-DD format</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Priority        — High / Medium / Low / Critical</t>
+          <t xml:space="preserve">  Date            — Task target/due date in YYYY-MM-DD format</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Assignee        — Person responsible</t>
+          <t xml:space="preserve">  Story Points    — Effort estimate (integer)</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  Status          — To Do / In Progress / Done / Blocked / In Review</t>
+          <t xml:space="preserve">  Priority        — High / Medium / Low / Critical</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="9" t="inlineStr">
         <is>
+          <t xml:space="preserve">  Assignee        — Person responsible</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  Status          — To Do / In Progress / Done / Blocked / In Review</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="9" t="inlineStr">
+        <is>
           <t xml:space="preserve">  Dependencies    — Optional free-text dependency notes</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="A23" s="9" t="inlineStr"/>
-    </row>
-    <row r="24">
-      <c r="A24" s="10" t="inlineStr">
+    <row r="25">
+      <c r="A25" s="9" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="10" t="inlineStr">
         <is>
           <t>Tips:</t>
-        </is>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Keep column order exactly as shown in the JIRA Data sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" s="9" t="inlineStr">
-        <is>
-          <t xml:space="preserve">  • Dates must be parseable by pandas (YYYY-MM-DD recommended).</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t xml:space="preserve">  • The 'Cost' column is ignored if present — safe to include or omit.</t>
+          <t xml:space="preserve">  • Keep column order exactly as shown in the JIRA Data sheet.</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • Dates must be parseable by pandas (YYYY-MM-DD recommended).</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  • The 'Cost' column is ignored if present — safe to include or omit.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="9" t="inlineStr">
         <is>
           <t xml:space="preserve">  • Remove these instruction rows before uploading.</t>
         </is>

</xml_diff>